<commit_message>
chore: 更新 now/MHXY.xlsx 数据
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/now/MHXY.xlsx
+++ b/now/MHXY.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="137">
   <si>
     <t>梦幻西游 · 支出明细表（黄色行为新增录入区）</t>
   </si>
@@ -79,6 +79,12 @@
   </si>
   <si>
     <t>主力账号</t>
+  </si>
+  <si>
+    <t>巫蛮儿</t>
+  </si>
+  <si>
+    <t>女儿村</t>
   </si>
   <si>
     <t/>
@@ -1701,9 +1707,15 @@
       <c r="A9" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="19"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="19"/>
+      <c r="B9" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="20">
+        <v>460</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" spans="1:4">
       <c r="A10" s="19" t="s">
@@ -1739,22 +1751,22 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:4">
       <c r="A14" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C14" s="22">
         <f>SUM(C4:C13)</f>
-        <v>2676.9</v>
+        <v>3136.9</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1" spans="1:4">
       <c r="A15" s="16" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -1762,136 +1774,136 @@
     </row>
     <row r="16" ht="16.5" customHeight="1" spans="1:4">
       <c r="A16" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C16" s="8">
         <v>30</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" ht="16.5" customHeight="1" spans="1:4">
       <c r="A17" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C17" s="8">
         <v>20</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" spans="1:4">
       <c r="A18" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C18" s="8">
         <v>5</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C19" s="8">
         <v>5</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C20" s="8">
         <v>5</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C21" s="8">
         <v>10</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C22" s="8">
         <v>25</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C23" s="8">
         <v>300</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" spans="1:4">
       <c r="A24" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C24" s="8">
         <v>125</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" spans="1:4">
       <c r="A25" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C25" s="20">
         <v>15</v>
@@ -1900,10 +1912,10 @@
     </row>
     <row r="26" ht="16.5" customHeight="1" spans="1:4">
       <c r="A26" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C26" s="20">
         <v>1.05</v>
@@ -1912,24 +1924,24 @@
     </row>
     <row r="27" ht="16.5" customHeight="1" spans="1:4">
       <c r="A27" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C27" s="20">
         <v>25</v>
       </c>
       <c r="D27" s="19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" spans="1:4">
       <c r="A28" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C28" s="20">
         <v>20</v>
@@ -1938,10 +1950,10 @@
     </row>
     <row r="29" ht="16.5" customHeight="1" spans="1:4">
       <c r="A29" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C29" s="20">
         <v>30</v>
@@ -1950,10 +1962,10 @@
     </row>
     <row r="30" ht="16.5" customHeight="1" spans="1:4">
       <c r="A30" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C30" s="20">
         <v>290</v>
@@ -1964,10 +1976,10 @@
     </row>
     <row r="31" ht="16.5" customHeight="1" spans="1:4">
       <c r="A31" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C31" s="20">
         <v>50</v>
@@ -1976,7 +1988,7 @@
     </row>
     <row r="32" ht="16.5" customHeight="1" spans="1:4">
       <c r="A32" s="19" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B32" s="21"/>
       <c r="C32" s="22"/>
@@ -1984,22 +1996,22 @@
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:4">
       <c r="A33" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C33" s="22">
         <f>SUM(C16:C31)</f>
         <v>956.05</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" ht="26" customHeight="1" spans="1:4">
       <c r="A34" s="16" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B34" s="17"/>
       <c r="C34" s="17"/>
@@ -2007,176 +2019,176 @@
     </row>
     <row r="35" ht="16.5" customHeight="1" spans="1:4">
       <c r="A35" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C35" s="8">
         <v>128</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="36" ht="16.5" customHeight="1" spans="1:4">
       <c r="A36" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C36" s="8">
         <v>140</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C37" s="8">
         <v>120</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" ht="16.5" customHeight="1" spans="1:4">
       <c r="A38" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C38" s="8">
         <v>168</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" ht="16.5" customHeight="1" spans="1:4">
       <c r="A39" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C39" s="8">
         <v>106</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="40" ht="16.5" customHeight="1" spans="1:4">
       <c r="A40" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C40" s="20">
         <v>68.25</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="41" ht="16.5" customHeight="1" spans="1:4">
       <c r="A41" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C41" s="20">
         <v>65</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42" ht="16.5" customHeight="1" spans="1:4">
       <c r="A42" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C42" s="20">
         <v>409</v>
       </c>
       <c r="D42" s="19" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" ht="16.5" customHeight="1" spans="1:4">
       <c r="A43" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C43" s="20">
         <v>177</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="44" ht="16.5" customHeight="1" spans="1:4">
       <c r="A44" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C44" s="20">
         <v>160</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" spans="1:4">
       <c r="A45" s="19" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C45" s="20">
         <v>240</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" ht="26" customHeight="1" spans="1:4">
       <c r="A46" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C46" s="22">
         <f>SUM(C35:C45)</f>
         <v>1781.25</v>
       </c>
       <c r="D46" s="21" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" spans="1:4">
       <c r="A47" s="16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B47" s="17"/>
       <c r="C47" s="17"/>
@@ -2184,49 +2196,49 @@
     </row>
     <row r="48" ht="16.5" customHeight="1" spans="1:4">
       <c r="A48" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C48" s="8">
         <v>20</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" ht="16.5" customHeight="1" spans="1:4">
       <c r="A49" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C49" s="8">
         <v>35</v>
       </c>
       <c r="D49" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" ht="16.5" customHeight="1" spans="1:4">
       <c r="A50" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C50" s="8">
         <v>40.5</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="51" ht="16.5" customHeight="1" spans="1:4">
       <c r="A51" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B51" s="19"/>
       <c r="C51" s="20"/>
@@ -2234,7 +2246,7 @@
     </row>
     <row r="52" ht="16.5" customHeight="1" spans="1:4">
       <c r="A52" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B52" s="19"/>
       <c r="C52" s="20"/>
@@ -2242,7 +2254,7 @@
     </row>
     <row r="53" ht="16.5" customHeight="1" spans="1:4">
       <c r="A53" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B53" s="19"/>
       <c r="C53" s="20"/>
@@ -2250,7 +2262,7 @@
     </row>
     <row r="54" ht="16.5" customHeight="1" spans="1:4">
       <c r="A54" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B54" s="19"/>
       <c r="C54" s="20"/>
@@ -2258,7 +2270,7 @@
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:4">
       <c r="A55" s="19" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B55" s="19"/>
       <c r="C55" s="20"/>
@@ -2266,44 +2278,44 @@
     </row>
     <row r="56" ht="15" spans="1:4">
       <c r="A56" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C56" s="22">
         <f>SUM(C48:C55)</f>
         <v>95.5</v>
       </c>
       <c r="D56" s="21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="57" ht="18" customHeight="1"/>
     <row r="58" ht="18" spans="1:4">
       <c r="A58" s="23" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B58" s="23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C58" s="11">
         <f>C14+C33+C46+C56</f>
-        <v>5509.7</v>
+        <v>5969.7</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59" ht="16.5" customHeight="1"/>
     <row r="60" ht="16.5" customHeight="1" spans="1:4">
       <c r="A60" s="14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="61" ht="16.5" spans="1:4">
       <c r="A61" s="14" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2334,15 +2346,15 @@
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -2353,7 +2365,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:4">
       <c r="A3" s="16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -2361,176 +2373,176 @@
     </row>
     <row r="4" ht="16.5" customHeight="1" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="8">
         <v>85.5</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" ht="16.5" customHeight="1" spans="1:4">
       <c r="A5" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="20">
         <v>161.5</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" ht="16.5" customHeight="1" spans="1:4">
       <c r="A6" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="20">
         <v>123.5</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" ht="16.5" customHeight="1" spans="1:4">
       <c r="A7" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C7" s="20">
         <v>9.5</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" ht="16.5" customHeight="1" spans="1:4">
       <c r="A8" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C8" s="20">
         <v>115</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" ht="16.5" customHeight="1" spans="1:4">
       <c r="A9" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C9" s="20">
         <v>9.5</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" ht="16.5" customHeight="1" spans="1:4">
       <c r="A10" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C10" s="20">
         <v>133</v>
       </c>
       <c r="D10" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" ht="16.5" customHeight="1" spans="1:4">
       <c r="A11" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C11" s="20">
         <v>66.5</v>
       </c>
       <c r="D11" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" ht="16.5" customHeight="1" spans="1:4">
       <c r="A12" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C12" s="20">
         <v>14.5</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" ht="16.5" customHeight="1" spans="1:4">
       <c r="A13" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C13" s="20">
         <v>14.5</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" spans="1:4">
       <c r="A14" s="19" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C14" s="20">
         <v>9.5</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:4">
       <c r="A15" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C15" s="22">
         <f>SUM(C4:C14)</f>
         <v>742.5</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1" spans="1:4">
       <c r="A16" s="16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -2538,289 +2550,289 @@
     </row>
     <row r="17" ht="16.5" customHeight="1" spans="1:4">
       <c r="A17" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C17" s="8">
         <v>202</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" ht="16.5" customHeight="1" spans="1:4">
       <c r="A18" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C18" s="8">
         <v>67.45</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C19" s="8">
         <v>67.45</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" ht="16.5" customHeight="1" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C20" s="8">
         <v>66.78</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="21" ht="16.5" customHeight="1" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C21" s="8">
         <v>66.78</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" ht="16.5" customHeight="1" spans="1:4">
       <c r="A22" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C22" s="20">
         <v>66.02</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" spans="1:4">
       <c r="A23" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C23" s="20">
         <v>65.55</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" spans="1:4">
       <c r="A24" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C24" s="20">
         <v>66.02</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" ht="16.5" customHeight="1" spans="1:4">
       <c r="A25" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C25" s="20">
         <v>69.2</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="26" ht="16.5" customHeight="1" spans="1:4">
       <c r="A26" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C26" s="20">
         <v>68</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" ht="16.5" customHeight="1" spans="1:4">
       <c r="A27" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C27" s="20">
         <v>41</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" ht="16.5" customHeight="1" spans="1:4">
       <c r="A28" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C28" s="20">
         <v>67.7</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="29" ht="16.5" customHeight="1" spans="1:4">
       <c r="A29" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C29" s="20">
         <v>68</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="30" ht="16.5" customHeight="1" spans="1:4">
       <c r="A30" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C30" s="20">
         <v>41.82</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:4">
       <c r="A31" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C31" s="20">
         <v>197</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:4">
       <c r="A32" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C32" s="20">
         <v>25.84</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" ht="16.5" spans="1:4">
       <c r="A33" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C33" s="20">
         <v>191.9</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" ht="16.5" spans="1:4">
       <c r="A34" s="19" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C34" s="20">
         <v>111</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" spans="1:4">
       <c r="A35" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C35" s="22">
         <f>SUM(C17:C34)</f>
         <v>1549.51</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" spans="1:4">
       <c r="A37" s="21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C37" s="22">
         <f>C15+C35</f>
         <v>2292.01</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="39" ht="16.5" spans="1:4">
       <c r="A39" s="14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2848,89 +2860,89 @@
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" ht="16.5" customHeight="1" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B3" s="5">
         <f>支出明细表!C58</f>
-        <v>5509.7</v>
+        <v>5969.7</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" spans="1:3">
       <c r="A4" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B4" s="8">
         <f>游戏变现收入明细表!C37</f>
         <v>2292.01</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" spans="1:3">
       <c r="A5" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B5" s="11">
         <f>B3-B4</f>
-        <v>3217.69</v>
+        <v>3677.69</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" spans="1:3">
       <c r="A7" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:3">
       <c r="A8" s="14" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:3">
       <c r="A9" s="14" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3">
       <c r="A10" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:3">
       <c r="A11" s="14" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:3">
       <c r="A12" s="14" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" ht="16.5" customHeight="1" spans="1:3">
       <c r="A14" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: 更新 now/MHXY.xlsx 记账数据
- 支出: 9月23点卡25
- 收入: 卖古代瑞兽胚子9.5

Co-Authored-By: AtomCode (glm5.3-flash) <noreply@atomgit.com>
</commit_message>
<xml_diff>
--- a/now/MHXY.xlsx
+++ b/now/MHXY.xlsx
@@ -1251,7 +1251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1821,51 +1821,47 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="21" t="inlineStr"/>
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>点卡相关</t>
+        </is>
+      </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
+          <t>9月23点卡</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="D34" s="21" t="n"/>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="21" t="inlineStr"/>
+      <c r="B35" s="21" t="inlineStr">
+        <is>
           <t>点卡小计</t>
         </is>
       </c>
-      <c r="C34" s="22">
-        <f>SUM(C16:C32)</f>
+      <c r="C35" s="22">
+        <f>SUM(C16:C33)</f>
         <v/>
       </c>
-      <c r="D34" s="21" t="inlineStr">
+      <c r="D35" s="21" t="inlineStr">
         <is>
           <t>全部点卡充值合计</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+    <row r="36" ht="16.5" customHeight="1">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>▌召唤兽采购</t>
         </is>
       </c>
-      <c r="B35" s="17" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="18" t="n"/>
-    </row>
-    <row r="36" ht="16.5" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>召唤兽采购</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>蓝书力宠画魂</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="n">
-        <v>128</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>力宠（已卖出）</t>
-        </is>
-      </c>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="18" t="n"/>
     </row>
     <row r="37" ht="16.5" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
@@ -1875,15 +1871,15 @@
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>力宠蝴蝶仙子</t>
+          <t>蓝书力宠画魂</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>力宠</t>
+          <t>力宠（已卖出）</t>
         </is>
       </c>
     </row>
@@ -1895,15 +1891,15 @@
       </c>
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>力宠吸血鬼</t>
+          <t>力宠蝴蝶仙子</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="D38" s="9" t="inlineStr">
         <is>
-          <t>力宠（已卖出）</t>
+          <t>力宠</t>
         </is>
       </c>
     </row>
@@ -1915,15 +1911,15 @@
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>力宠龙鲤</t>
+          <t>力宠吸血鬼</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
-        <v>168</v>
+        <v>120</v>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>力宠 （已卖出）</t>
+          <t>力宠（已卖出）</t>
         </is>
       </c>
     </row>
@@ -1935,35 +1931,35 @@
       </c>
       <c r="B40" s="9" t="inlineStr">
         <is>
+          <t>力宠龙鲤</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n">
+        <v>168</v>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>力宠 （已卖出）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>召唤兽采购</t>
+        </is>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
           <t>购入法宠</t>
         </is>
       </c>
-      <c r="C40" s="8" t="n">
+      <c r="C41" s="8" t="n">
         <v>106</v>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D41" s="9" t="inlineStr">
         <is>
           <t>法宠（后续卖出）</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16.5" customHeight="1">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>召唤兽采购</t>
-        </is>
-      </c>
-      <c r="B41" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">79龙鲤 </t>
-        </is>
-      </c>
-      <c r="C41" s="20" t="n">
-        <v>68.25</v>
-      </c>
-      <c r="D41" s="9" t="inlineStr">
-        <is>
-          <t>力宠</t>
         </is>
       </c>
     </row>
@@ -1975,11 +1971,11 @@
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>79龙鲤 2</t>
+          <t xml:space="preserve">79龙鲤 </t>
         </is>
       </c>
       <c r="C42" s="20" t="n">
-        <v>65</v>
+        <v>68.25</v>
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
@@ -1995,15 +1991,15 @@
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>须弥画魂高魔心带套0903</t>
+          <t>79龙鲤 2</t>
         </is>
       </c>
       <c r="C43" s="20" t="n">
-        <v>409</v>
-      </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>法宠</t>
+        <v>65</v>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>力宠</t>
         </is>
       </c>
     </row>
@@ -2015,15 +2011,15 @@
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">龙鲤0908 </t>
+          <t>须弥画魂高魔心带套0903</t>
         </is>
       </c>
       <c r="C44" s="20" t="n">
-        <v>177</v>
-      </c>
-      <c r="D44" s="9" t="inlineStr">
-        <is>
-          <t>力宠</t>
+        <v>409</v>
+      </c>
+      <c r="D44" s="19" t="inlineStr">
+        <is>
+          <t>法宠</t>
         </is>
       </c>
     </row>
@@ -2035,11 +2031,11 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>三技能女娲0908</t>
+          <t xml:space="preserve">龙鲤0908 </t>
         </is>
       </c>
       <c r="C45" s="20" t="n">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
@@ -2055,15 +2051,15 @@
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>雷鸟人须弥 9月20</t>
+          <t>三技能女娲0908</t>
         </is>
       </c>
       <c r="C46" s="20" t="n">
-        <v>210</v>
+        <v>160</v>
       </c>
       <c r="D46" s="9" t="inlineStr">
         <is>
-          <t>须弥法宠</t>
+          <t>力宠</t>
         </is>
       </c>
     </row>
@@ -2075,64 +2071,64 @@
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
+          <t>雷鸟人须弥 9月20</t>
+        </is>
+      </c>
+      <c r="C47" s="20" t="n">
+        <v>210</v>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>须弥法宠</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="26" customHeight="1">
+      <c r="A48" s="19" t="inlineStr">
+        <is>
+          <t>召唤兽采购</t>
+        </is>
+      </c>
+      <c r="B48" s="19" t="inlineStr">
+        <is>
           <t>雷鸟人须弥 9月11</t>
         </is>
       </c>
-      <c r="C47" s="20" t="n">
+      <c r="C48" s="20" t="n">
         <v>240</v>
       </c>
-      <c r="D47" s="9" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>须弥法宠</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="21" t="inlineStr"/>
-      <c r="B48" s="21" t="inlineStr">
+    <row r="49" ht="16.5" customHeight="1">
+      <c r="A49" s="21" t="inlineStr"/>
+      <c r="B49" s="21" t="inlineStr">
         <is>
           <t>购宠小计</t>
         </is>
       </c>
-      <c r="C48" s="22">
-        <f>SUM(C36:C47)</f>
+      <c r="C49" s="22">
+        <f>SUM(C37:C48)</f>
         <v/>
       </c>
-      <c r="D48" s="21" t="inlineStr">
+      <c r="D49" s="21" t="inlineStr">
         <is>
           <t>宠物采购总花费</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1">
-      <c r="A49" s="16" t="inlineStr">
+    <row r="50" ht="16.5" customHeight="1">
+      <c r="A50" s="16" t="inlineStr">
         <is>
           <t>▌装备采购</t>
         </is>
       </c>
-      <c r="B49" s="17" t="n"/>
-      <c r="C49" s="17" t="n"/>
-      <c r="D49" s="18" t="n"/>
-    </row>
-    <row r="50" ht="16.5" customHeight="1">
-      <c r="A50" s="9" t="inlineStr">
-        <is>
-          <t>装备采购</t>
-        </is>
-      </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>主号武器</t>
-        </is>
-      </c>
-      <c r="C50" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D50" s="9" t="inlineStr">
-        <is>
-          <t>主力角色装备</t>
-        </is>
-      </c>
+      <c r="B50" s="17" t="n"/>
+      <c r="C50" s="17" t="n"/>
+      <c r="D50" s="18" t="n"/>
     </row>
     <row r="51" ht="16.5" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
@@ -2142,11 +2138,11 @@
       </c>
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>主号鞋子</t>
+          <t>主号武器</t>
         </is>
       </c>
       <c r="C51" s="8" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
@@ -2162,35 +2158,35 @@
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
+          <t>主号鞋子</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>主力角色装备</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16.5" customHeight="1">
+      <c r="A53" s="9" t="inlineStr">
+        <is>
+          <t>装备采购</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
           <t>4 角色 100 级国标武器</t>
         </is>
       </c>
-      <c r="C52" s="8" t="n">
+      <c r="C53" s="8" t="n">
         <v>40.5</v>
       </c>
-      <c r="D52" s="9" t="inlineStr">
+      <c r="D53" s="9" t="inlineStr">
         <is>
           <t>其余小号武器</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="16.5" customHeight="1">
-      <c r="A53" s="19" t="inlineStr">
-        <is>
-          <t>装备采购</t>
-        </is>
-      </c>
-      <c r="B53" s="19" t="inlineStr">
-        <is>
-          <t>后排灵饰109</t>
-        </is>
-      </c>
-      <c r="C53" s="20" t="n">
-        <v>109</v>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>装备采购</t>
         </is>
       </c>
     </row>
@@ -2202,11 +2198,11 @@
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>风伯套装48</t>
+          <t>后排灵饰109</t>
         </is>
       </c>
       <c r="C54" s="20" t="n">
-        <v>48</v>
+        <v>109</v>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
@@ -2222,11 +2218,11 @@
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>吸血鬼鞋子（套牢）</t>
+          <t>风伯套装48</t>
         </is>
       </c>
       <c r="C55" s="20" t="n">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
@@ -2242,11 +2238,11 @@
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>国标武器</t>
+          <t>吸血鬼鞋子（套牢）</t>
         </is>
       </c>
       <c r="C56" s="20" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
@@ -2260,55 +2256,75 @@
           <t>装备采购</t>
         </is>
       </c>
-      <c r="B57" s="19" t="n"/>
-      <c r="C57" s="20" t="n"/>
-      <c r="D57" s="19" t="n"/>
+      <c r="B57" s="19" t="inlineStr">
+        <is>
+          <t>国标武器</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>装备采购</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1">
-      <c r="A58" s="21" t="inlineStr"/>
-      <c r="B58" s="21" t="inlineStr">
+      <c r="A58" s="19" t="inlineStr">
+        <is>
+          <t>装备采购</t>
+        </is>
+      </c>
+      <c r="B58" s="19" t="n"/>
+      <c r="C58" s="20" t="n"/>
+      <c r="D58" s="19" t="n"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="21" t="inlineStr"/>
+      <c r="B59" s="21" t="inlineStr">
         <is>
           <t>装备小计</t>
         </is>
       </c>
-      <c r="C58" s="22">
-        <f>SUM(C50:C57)</f>
+      <c r="C59" s="22">
+        <f>SUM(C51:C58)</f>
         <v/>
       </c>
-      <c r="D58" s="21" t="inlineStr">
+      <c r="D59" s="21" t="inlineStr">
         <is>
           <t>装备总花费</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="18" customHeight="1"/>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="24" t="inlineStr"/>
-      <c r="B60" s="24" t="inlineStr">
+    <row r="60" ht="18" customHeight="1"/>
+    <row r="61" ht="16.5" customHeight="1">
+      <c r="A61" s="24" t="n"/>
+      <c r="B61" s="24" t="inlineStr">
         <is>
           <t>全部支出合计</t>
         </is>
       </c>
-      <c r="C60" s="11">
-        <f>C14+C34+C48+C58</f>
+      <c r="C61" s="11">
+        <f>C14+C35+C49+C59</f>
         <v/>
       </c>
-      <c r="D60" s="24" t="inlineStr">
+      <c r="D61" s="24" t="inlineStr">
         <is>
           <t>所有板块总支出</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="16.5" customHeight="1"/>
-    <row r="62" ht="16.5" customHeight="1">
-      <c r="A62" s="14" t="inlineStr">
-        <is>
-          <t>📌 操作说明：在黄色底纹行录入新支出，金额填入 C 列，小计和合计自动更新。</t>
-        </is>
-      </c>
-    </row>
+    <row r="62" ht="16.5" customHeight="1"/>
     <row r="63" ht="16.5" customHeight="1">
       <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>📌 操作说明：在黄色底纹行录入新支出，金额填入 C 列，小计和合计自动更新。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
         <is>
           <t>📌 如需更多行：右键插入行 → 从上方黄色行复制格式即可。</t>
         </is>
@@ -2317,11 +2333,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="A62:D62"/>
+    <mergeCell ref="A50:D50"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A49:D49"/>
+    <mergeCell ref="A63:D63"/>
+    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2333,7 +2349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3005,41 +3021,57 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="n"/>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
+        <is>
+          <t>物资变现</t>
+        </is>
+      </c>
+      <c r="B36" s="19" t="inlineStr">
+        <is>
+          <t>卖古代瑞兽胚子 9月23</t>
+        </is>
+      </c>
+      <c r="C36" s="19" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="D36" s="19" t="n"/>
+    </row>
+    <row r="37" ht="16.5" customHeight="1">
+      <c r="A37" s="23" t="n"/>
+      <c r="B37" s="23" t="inlineStr">
         <is>
           <t>物资小计</t>
         </is>
       </c>
-      <c r="C36" s="23">
-        <f>SUM(C17:C35)</f>
+      <c r="C37" s="23">
+        <f>SUM(C17:C36)</f>
         <v/>
       </c>
-      <c r="D36" s="23" t="n"/>
-    </row>
-    <row r="37" ht="16.5" customHeight="1">
-      <c r="A37" s="21" t="inlineStr"/>
-      <c r="B37" s="21" t="n"/>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D37" s="23" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr"/>
+      <c r="B38" s="21" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="21" t="inlineStr">
         <is>
           <t>所有回款合计</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" t="inlineStr">
+    <row r="39" ht="16.5" customHeight="1">
+      <c r="B39" t="inlineStr">
         <is>
           <t>全部变现总收入</t>
         </is>
       </c>
-      <c r="C38">
-        <f>C15+C36</f>
+      <c r="C39">
+        <f>C15+C37</f>
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>📌 操作说明：在黄色底纹行录入新收入，金额填入 C 列，小计和合计自动更新。</t>
         </is>
@@ -3048,9 +3080,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A40:D40"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A16:D16"/>
-    <mergeCell ref="A39:D39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>